<commit_message>
Updated Manu Script as of 9/15/2026
</commit_message>
<xml_diff>
--- a/REDCap/Input Sheets/Excel Sheets/C-LR_Low Res- TEST.xlsx
+++ b/REDCap/Input Sheets/Excel Sheets/C-LR_Low Res- TEST.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nvuko\CBOTH_Summer_2026\REDCap\Input Sheets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nvuko\CBOTH_Summer_2026\REDCap\Input Sheets\Excel Sheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E51512A6-8107-449C-A512-7719810702AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EF1F6D7-D762-43FD-B643-D537234B5AB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{115E3380-263E-460B-BE56-F11D0EF2B802}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{115E3380-263E-460B-BE56-F11D0EF2B802}"/>
   </bookViews>
   <sheets>
     <sheet name="C-TST 01" sheetId="1" r:id="rId1"/>
@@ -932,50 +932,8 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="20" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="16" fontId="20" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
@@ -1003,6 +961,48 @@
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="20" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="16" fontId="20" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1353,23 +1353,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:52" ht="25.8">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="45" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="58"/>
-      <c r="C1" s="58"/>
-      <c r="D1" s="58"/>
-      <c r="E1" s="58"/>
-      <c r="F1" s="59"/>
-      <c r="G1" s="57" t="s">
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="45" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="58"/>
-      <c r="I1" s="58"/>
-      <c r="J1" s="58"/>
-      <c r="K1" s="58"/>
-      <c r="L1" s="58"/>
-      <c r="M1" s="59"/>
+      <c r="H1" s="46"/>
+      <c r="I1" s="46"/>
+      <c r="J1" s="46"/>
+      <c r="K1" s="46"/>
+      <c r="L1" s="46"/>
+      <c r="M1" s="47"/>
       <c r="N1" s="29"/>
       <c r="O1" s="29"/>
       <c r="P1" s="29"/>
@@ -1411,19 +1411,19 @@
       <c r="AZ1" s="2"/>
     </row>
     <row r="2" spans="1:52" ht="26.4" thickBot="1">
-      <c r="A2" s="60"/>
-      <c r="B2" s="61"/>
-      <c r="C2" s="61"/>
-      <c r="D2" s="61"/>
-      <c r="E2" s="61"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="60"/>
-      <c r="H2" s="61"/>
-      <c r="I2" s="61"/>
-      <c r="J2" s="61"/>
-      <c r="K2" s="61"/>
-      <c r="L2" s="61"/>
-      <c r="M2" s="62"/>
+      <c r="A2" s="48"/>
+      <c r="B2" s="49"/>
+      <c r="C2" s="49"/>
+      <c r="D2" s="49"/>
+      <c r="E2" s="49"/>
+      <c r="F2" s="50"/>
+      <c r="G2" s="48"/>
+      <c r="H2" s="49"/>
+      <c r="I2" s="49"/>
+      <c r="J2" s="49"/>
+      <c r="K2" s="49"/>
+      <c r="L2" s="49"/>
+      <c r="M2" s="50"/>
       <c r="N2" s="30"/>
       <c r="O2" s="30"/>
       <c r="P2" s="30"/>
@@ -1485,37 +1485,37 @@
       <c r="R3" s="31"/>
       <c r="T3" s="31"/>
       <c r="U3" s="31"/>
-      <c r="V3" s="63"/>
-      <c r="W3" s="63"/>
-      <c r="X3" s="54"/>
-      <c r="Y3" s="54"/>
-      <c r="Z3" s="54"/>
-      <c r="AA3" s="54"/>
-      <c r="AB3" s="54"/>
-      <c r="AC3" s="54"/>
-      <c r="AD3" s="54"/>
-      <c r="AE3" s="54"/>
-      <c r="AF3" s="54"/>
-      <c r="AG3" s="54"/>
-      <c r="AH3" s="51"/>
-      <c r="AI3" s="51"/>
-      <c r="AJ3" s="51"/>
-      <c r="AK3" s="51"/>
-      <c r="AL3" s="51"/>
-      <c r="AM3" s="51"/>
-      <c r="AN3" s="51"/>
-      <c r="AO3" s="51"/>
-      <c r="AP3" s="51"/>
-      <c r="AQ3" s="51"/>
-      <c r="AR3" s="51"/>
-      <c r="AS3" s="51"/>
-      <c r="AT3" s="51"/>
-      <c r="AU3" s="51"/>
-      <c r="AV3" s="51"/>
-      <c r="AW3" s="51"/>
-      <c r="AX3" s="51"/>
-      <c r="AY3" s="51"/>
-      <c r="AZ3" s="51"/>
+      <c r="V3" s="51"/>
+      <c r="W3" s="51"/>
+      <c r="X3" s="44"/>
+      <c r="Y3" s="44"/>
+      <c r="Z3" s="44"/>
+      <c r="AA3" s="44"/>
+      <c r="AB3" s="44"/>
+      <c r="AC3" s="44"/>
+      <c r="AD3" s="44"/>
+      <c r="AE3" s="44"/>
+      <c r="AF3" s="44"/>
+      <c r="AG3" s="44"/>
+      <c r="AH3" s="58"/>
+      <c r="AI3" s="58"/>
+      <c r="AJ3" s="58"/>
+      <c r="AK3" s="58"/>
+      <c r="AL3" s="58"/>
+      <c r="AM3" s="58"/>
+      <c r="AN3" s="58"/>
+      <c r="AO3" s="58"/>
+      <c r="AP3" s="58"/>
+      <c r="AQ3" s="58"/>
+      <c r="AR3" s="58"/>
+      <c r="AS3" s="58"/>
+      <c r="AT3" s="58"/>
+      <c r="AU3" s="58"/>
+      <c r="AV3" s="58"/>
+      <c r="AW3" s="58"/>
+      <c r="AX3" s="58"/>
+      <c r="AY3" s="58"/>
+      <c r="AZ3" s="58"/>
     </row>
     <row r="4" spans="1:52" ht="43.8" thickBot="1">
       <c r="A4" s="32" t="s">
@@ -1529,10 +1529,10 @@
       <c r="E4" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="48">
+      <c r="F4" s="56">
         <v>1</v>
       </c>
-      <c r="G4" s="49"/>
+      <c r="G4" s="57"/>
       <c r="H4" s="31"/>
       <c r="I4" s="31"/>
       <c r="J4" s="30"/>
@@ -1549,37 +1549,37 @@
       <c r="S4" s="37"/>
       <c r="T4" s="37"/>
       <c r="U4" s="31"/>
-      <c r="V4" s="63"/>
-      <c r="W4" s="63"/>
-      <c r="X4" s="54"/>
-      <c r="Y4" s="54"/>
-      <c r="Z4" s="54"/>
-      <c r="AA4" s="54"/>
-      <c r="AB4" s="54"/>
-      <c r="AC4" s="54"/>
-      <c r="AD4" s="54"/>
-      <c r="AE4" s="54"/>
-      <c r="AF4" s="54"/>
-      <c r="AG4" s="54"/>
-      <c r="AH4" s="51"/>
-      <c r="AI4" s="51"/>
-      <c r="AJ4" s="51"/>
-      <c r="AK4" s="51"/>
-      <c r="AL4" s="51"/>
-      <c r="AM4" s="51"/>
-      <c r="AN4" s="51"/>
-      <c r="AO4" s="51"/>
-      <c r="AP4" s="51"/>
-      <c r="AQ4" s="51"/>
-      <c r="AR4" s="51"/>
-      <c r="AS4" s="51"/>
-      <c r="AT4" s="51"/>
-      <c r="AU4" s="51"/>
-      <c r="AV4" s="51"/>
-      <c r="AW4" s="51"/>
-      <c r="AX4" s="51"/>
-      <c r="AY4" s="51"/>
-      <c r="AZ4" s="51"/>
+      <c r="V4" s="51"/>
+      <c r="W4" s="51"/>
+      <c r="X4" s="44"/>
+      <c r="Y4" s="44"/>
+      <c r="Z4" s="44"/>
+      <c r="AA4" s="44"/>
+      <c r="AB4" s="44"/>
+      <c r="AC4" s="44"/>
+      <c r="AD4" s="44"/>
+      <c r="AE4" s="44"/>
+      <c r="AF4" s="44"/>
+      <c r="AG4" s="44"/>
+      <c r="AH4" s="58"/>
+      <c r="AI4" s="58"/>
+      <c r="AJ4" s="58"/>
+      <c r="AK4" s="58"/>
+      <c r="AL4" s="58"/>
+      <c r="AM4" s="58"/>
+      <c r="AN4" s="58"/>
+      <c r="AO4" s="58"/>
+      <c r="AP4" s="58"/>
+      <c r="AQ4" s="58"/>
+      <c r="AR4" s="58"/>
+      <c r="AS4" s="58"/>
+      <c r="AT4" s="58"/>
+      <c r="AU4" s="58"/>
+      <c r="AV4" s="58"/>
+      <c r="AW4" s="58"/>
+      <c r="AX4" s="58"/>
+      <c r="AY4" s="58"/>
+      <c r="AZ4" s="58"/>
     </row>
     <row r="5" spans="1:52" ht="26.4" thickBot="1">
       <c r="A5" s="32" t="s">
@@ -1593,19 +1593,19 @@
       <c r="E5" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="55" t="s">
+      <c r="F5" s="54" t="s">
         <v>116</v>
       </c>
-      <c r="G5" s="56"/>
+      <c r="G5" s="55"/>
       <c r="H5" s="31"/>
       <c r="I5" s="31"/>
       <c r="J5" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="K5" s="48">
+      <c r="K5" s="56">
         <v>0.5</v>
       </c>
-      <c r="L5" s="49"/>
+      <c r="L5" s="57"/>
       <c r="M5" s="31"/>
       <c r="N5" s="32" t="s">
         <v>5</v>
@@ -1657,10 +1657,10 @@
       <c r="A6" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="46">
+      <c r="B6" s="61">
         <v>46225</v>
       </c>
-      <c r="C6" s="47"/>
+      <c r="C6" s="62"/>
       <c r="D6" s="33"/>
       <c r="E6" s="33"/>
       <c r="F6" s="31"/>
@@ -1670,10 +1670,10 @@
       <c r="J6" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="K6" s="48">
+      <c r="K6" s="56">
         <v>2</v>
       </c>
-      <c r="L6" s="49"/>
+      <c r="L6" s="57"/>
       <c r="M6" s="31"/>
       <c r="N6" s="32" t="s">
         <v>9</v>
@@ -1729,7 +1729,7 @@
         <v>63.22</v>
       </c>
       <c r="C7" s="40">
-        <v>41.34</v>
+        <v>45</v>
       </c>
       <c r="D7" s="33"/>
       <c r="E7" s="33"/>
@@ -1792,7 +1792,7 @@
         <v>63.22</v>
       </c>
       <c r="C8" s="42">
-        <v>41.34</v>
+        <v>45</v>
       </c>
       <c r="D8" s="33"/>
       <c r="E8" s="33"/>
@@ -2119,70 +2119,70 @@
       <c r="F12" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="G12" s="44" t="s">
+      <c r="G12" s="59" t="s">
         <v>19</v>
       </c>
-      <c r="H12" s="44"/>
-      <c r="I12" s="44"/>
-      <c r="J12" s="44"/>
-      <c r="K12" s="44"/>
+      <c r="H12" s="59"/>
+      <c r="I12" s="59"/>
+      <c r="J12" s="59"/>
+      <c r="K12" s="59"/>
       <c r="L12" s="8" t="s">
         <v>20</v>
       </c>
       <c r="M12" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="N12" s="45" t="s">
+      <c r="N12" s="60" t="s">
         <v>22</v>
       </c>
-      <c r="O12" s="45"/>
-      <c r="P12" s="45"/>
-      <c r="Q12" s="45"/>
-      <c r="R12" s="50" t="s">
+      <c r="O12" s="60"/>
+      <c r="P12" s="60"/>
+      <c r="Q12" s="60"/>
+      <c r="R12" s="63" t="s">
         <v>23</v>
       </c>
-      <c r="S12" s="50"/>
-      <c r="T12" s="50"/>
-      <c r="U12" s="50"/>
-      <c r="V12" s="50"/>
-      <c r="W12" s="50"/>
-      <c r="X12" s="50"/>
-      <c r="Y12" s="50"/>
-      <c r="Z12" s="50"/>
-      <c r="AA12" s="44" t="s">
+      <c r="S12" s="63"/>
+      <c r="T12" s="63"/>
+      <c r="U12" s="63"/>
+      <c r="V12" s="63"/>
+      <c r="W12" s="63"/>
+      <c r="X12" s="63"/>
+      <c r="Y12" s="63"/>
+      <c r="Z12" s="63"/>
+      <c r="AA12" s="59" t="s">
         <v>24</v>
       </c>
-      <c r="AB12" s="44"/>
-      <c r="AC12" s="44"/>
-      <c r="AD12" s="44"/>
-      <c r="AE12" s="44" t="s">
+      <c r="AB12" s="59"/>
+      <c r="AC12" s="59"/>
+      <c r="AD12" s="59"/>
+      <c r="AE12" s="59" t="s">
         <v>25</v>
       </c>
-      <c r="AF12" s="44"/>
-      <c r="AG12" s="44"/>
-      <c r="AH12" s="44"/>
-      <c r="AI12" s="45" t="s">
+      <c r="AF12" s="59"/>
+      <c r="AG12" s="59"/>
+      <c r="AH12" s="59"/>
+      <c r="AI12" s="60" t="s">
         <v>26</v>
       </c>
-      <c r="AJ12" s="45"/>
-      <c r="AK12" s="45"/>
-      <c r="AL12" s="45"/>
-      <c r="AM12" s="45"/>
-      <c r="AN12" s="45"/>
-      <c r="AO12" s="45"/>
-      <c r="AP12" s="45"/>
-      <c r="AQ12" s="45"/>
-      <c r="AR12" s="45"/>
-      <c r="AS12" s="45"/>
-      <c r="AT12" s="45"/>
-      <c r="AU12" s="45"/>
-      <c r="AV12" s="45"/>
-      <c r="AW12" s="45"/>
-      <c r="AX12" s="45"/>
-      <c r="AY12" s="45" t="s">
+      <c r="AJ12" s="60"/>
+      <c r="AK12" s="60"/>
+      <c r="AL12" s="60"/>
+      <c r="AM12" s="60"/>
+      <c r="AN12" s="60"/>
+      <c r="AO12" s="60"/>
+      <c r="AP12" s="60"/>
+      <c r="AQ12" s="60"/>
+      <c r="AR12" s="60"/>
+      <c r="AS12" s="60"/>
+      <c r="AT12" s="60"/>
+      <c r="AU12" s="60"/>
+      <c r="AV12" s="60"/>
+      <c r="AW12" s="60"/>
+      <c r="AX12" s="60"/>
+      <c r="AY12" s="60" t="s">
         <v>27</v>
       </c>
-      <c r="AZ12" s="45"/>
+      <c r="AZ12" s="60"/>
     </row>
     <row r="13" spans="1:52" ht="15.6">
       <c r="A13" s="8"/>
@@ -3874,13 +3874,34 @@
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="AY12:AZ12"/>
-    <mergeCell ref="AE12:AH12"/>
-    <mergeCell ref="G12:K12"/>
-    <mergeCell ref="N12:Q12"/>
-    <mergeCell ref="R12:Z12"/>
-    <mergeCell ref="AA12:AD12"/>
-    <mergeCell ref="AI12:AX12"/>
+    <mergeCell ref="A1:F2"/>
+    <mergeCell ref="G1:M2"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="K6:L6"/>
+    <mergeCell ref="AB3:AB4"/>
+    <mergeCell ref="V3:V4"/>
+    <mergeCell ref="W3:W4"/>
+    <mergeCell ref="X3:X4"/>
+    <mergeCell ref="Y3:Y4"/>
+    <mergeCell ref="Z3:Z4"/>
+    <mergeCell ref="AA3:AA4"/>
+    <mergeCell ref="AN3:AN4"/>
+    <mergeCell ref="AC3:AC4"/>
+    <mergeCell ref="AD3:AD4"/>
+    <mergeCell ref="AE3:AE4"/>
+    <mergeCell ref="AF3:AF4"/>
+    <mergeCell ref="AG3:AG4"/>
+    <mergeCell ref="AH3:AH4"/>
+    <mergeCell ref="AI3:AI4"/>
+    <mergeCell ref="AJ3:AJ4"/>
+    <mergeCell ref="AK3:AK4"/>
+    <mergeCell ref="AL3:AL4"/>
+    <mergeCell ref="AM3:AM4"/>
     <mergeCell ref="AZ3:AZ4"/>
     <mergeCell ref="AO3:AO4"/>
     <mergeCell ref="AP3:AP4"/>
@@ -3893,34 +3914,13 @@
     <mergeCell ref="AW3:AW4"/>
     <mergeCell ref="AX3:AX4"/>
     <mergeCell ref="AY3:AY4"/>
-    <mergeCell ref="AN3:AN4"/>
-    <mergeCell ref="AC3:AC4"/>
-    <mergeCell ref="AD3:AD4"/>
-    <mergeCell ref="AE3:AE4"/>
-    <mergeCell ref="AF3:AF4"/>
-    <mergeCell ref="AG3:AG4"/>
-    <mergeCell ref="AH3:AH4"/>
-    <mergeCell ref="AI3:AI4"/>
-    <mergeCell ref="AJ3:AJ4"/>
-    <mergeCell ref="AK3:AK4"/>
-    <mergeCell ref="AL3:AL4"/>
-    <mergeCell ref="AM3:AM4"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="K6:L6"/>
-    <mergeCell ref="AB3:AB4"/>
-    <mergeCell ref="V3:V4"/>
-    <mergeCell ref="W3:W4"/>
-    <mergeCell ref="X3:X4"/>
-    <mergeCell ref="Y3:Y4"/>
-    <mergeCell ref="Z3:Z4"/>
-    <mergeCell ref="AA3:AA4"/>
-    <mergeCell ref="A1:F2"/>
-    <mergeCell ref="G1:M2"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="AY12:AZ12"/>
+    <mergeCell ref="AE12:AH12"/>
+    <mergeCell ref="G12:K12"/>
+    <mergeCell ref="N12:Q12"/>
+    <mergeCell ref="R12:Z12"/>
+    <mergeCell ref="AA12:AD12"/>
+    <mergeCell ref="AI12:AX12"/>
   </mergeCells>
   <phoneticPr fontId="24" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3942,23 +3942,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:52" ht="25.8">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="45" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="58"/>
-      <c r="C1" s="58"/>
-      <c r="D1" s="58"/>
-      <c r="E1" s="58"/>
-      <c r="F1" s="59"/>
-      <c r="G1" s="57" t="s">
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="45" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="58"/>
-      <c r="I1" s="58"/>
-      <c r="J1" s="58"/>
-      <c r="K1" s="58"/>
-      <c r="L1" s="58"/>
-      <c r="M1" s="59"/>
+      <c r="H1" s="46"/>
+      <c r="I1" s="46"/>
+      <c r="J1" s="46"/>
+      <c r="K1" s="46"/>
+      <c r="L1" s="46"/>
+      <c r="M1" s="47"/>
       <c r="N1" s="29"/>
       <c r="O1" s="29"/>
       <c r="P1" s="29"/>
@@ -4000,19 +4000,19 @@
       <c r="AZ1" s="2"/>
     </row>
     <row r="2" spans="1:52" ht="26.4" thickBot="1">
-      <c r="A2" s="60"/>
-      <c r="B2" s="61"/>
-      <c r="C2" s="61"/>
-      <c r="D2" s="61"/>
-      <c r="E2" s="61"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="60"/>
-      <c r="H2" s="61"/>
-      <c r="I2" s="61"/>
-      <c r="J2" s="61"/>
-      <c r="K2" s="61"/>
-      <c r="L2" s="61"/>
-      <c r="M2" s="62"/>
+      <c r="A2" s="48"/>
+      <c r="B2" s="49"/>
+      <c r="C2" s="49"/>
+      <c r="D2" s="49"/>
+      <c r="E2" s="49"/>
+      <c r="F2" s="50"/>
+      <c r="G2" s="48"/>
+      <c r="H2" s="49"/>
+      <c r="I2" s="49"/>
+      <c r="J2" s="49"/>
+      <c r="K2" s="49"/>
+      <c r="L2" s="49"/>
+      <c r="M2" s="50"/>
       <c r="N2" s="30"/>
       <c r="O2" s="30"/>
       <c r="P2" s="30"/>
@@ -4074,37 +4074,37 @@
       <c r="R3" s="31"/>
       <c r="T3" s="31"/>
       <c r="U3" s="31"/>
-      <c r="V3" s="63"/>
-      <c r="W3" s="63"/>
-      <c r="X3" s="54"/>
-      <c r="Y3" s="54"/>
-      <c r="Z3" s="54"/>
-      <c r="AA3" s="54"/>
-      <c r="AB3" s="54"/>
-      <c r="AC3" s="54"/>
-      <c r="AD3" s="54"/>
-      <c r="AE3" s="54"/>
-      <c r="AF3" s="54"/>
-      <c r="AG3" s="54"/>
-      <c r="AH3" s="51"/>
-      <c r="AI3" s="51"/>
-      <c r="AJ3" s="51"/>
-      <c r="AK3" s="51"/>
-      <c r="AL3" s="51"/>
-      <c r="AM3" s="51"/>
-      <c r="AN3" s="51"/>
-      <c r="AO3" s="51"/>
-      <c r="AP3" s="51"/>
-      <c r="AQ3" s="51"/>
-      <c r="AR3" s="51"/>
-      <c r="AS3" s="51"/>
-      <c r="AT3" s="51"/>
-      <c r="AU3" s="51"/>
-      <c r="AV3" s="51"/>
-      <c r="AW3" s="51"/>
-      <c r="AX3" s="51"/>
-      <c r="AY3" s="51"/>
-      <c r="AZ3" s="51"/>
+      <c r="V3" s="51"/>
+      <c r="W3" s="51"/>
+      <c r="X3" s="44"/>
+      <c r="Y3" s="44"/>
+      <c r="Z3" s="44"/>
+      <c r="AA3" s="44"/>
+      <c r="AB3" s="44"/>
+      <c r="AC3" s="44"/>
+      <c r="AD3" s="44"/>
+      <c r="AE3" s="44"/>
+      <c r="AF3" s="44"/>
+      <c r="AG3" s="44"/>
+      <c r="AH3" s="58"/>
+      <c r="AI3" s="58"/>
+      <c r="AJ3" s="58"/>
+      <c r="AK3" s="58"/>
+      <c r="AL3" s="58"/>
+      <c r="AM3" s="58"/>
+      <c r="AN3" s="58"/>
+      <c r="AO3" s="58"/>
+      <c r="AP3" s="58"/>
+      <c r="AQ3" s="58"/>
+      <c r="AR3" s="58"/>
+      <c r="AS3" s="58"/>
+      <c r="AT3" s="58"/>
+      <c r="AU3" s="58"/>
+      <c r="AV3" s="58"/>
+      <c r="AW3" s="58"/>
+      <c r="AX3" s="58"/>
+      <c r="AY3" s="58"/>
+      <c r="AZ3" s="58"/>
     </row>
     <row r="4" spans="1:52" ht="43.8" thickBot="1">
       <c r="A4" s="32" t="s">
@@ -4118,10 +4118,10 @@
       <c r="E4" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="48">
+      <c r="F4" s="56">
         <v>0</v>
       </c>
-      <c r="G4" s="49"/>
+      <c r="G4" s="57"/>
       <c r="H4" s="31"/>
       <c r="I4" s="31"/>
       <c r="J4" s="30"/>
@@ -4142,37 +4142,37 @@
         <v>108</v>
       </c>
       <c r="U4" s="31"/>
-      <c r="V4" s="63"/>
-      <c r="W4" s="63"/>
-      <c r="X4" s="54"/>
-      <c r="Y4" s="54"/>
-      <c r="Z4" s="54"/>
-      <c r="AA4" s="54"/>
-      <c r="AB4" s="54"/>
-      <c r="AC4" s="54"/>
-      <c r="AD4" s="54"/>
-      <c r="AE4" s="54"/>
-      <c r="AF4" s="54"/>
-      <c r="AG4" s="54"/>
-      <c r="AH4" s="51"/>
-      <c r="AI4" s="51"/>
-      <c r="AJ4" s="51"/>
-      <c r="AK4" s="51"/>
-      <c r="AL4" s="51"/>
-      <c r="AM4" s="51"/>
-      <c r="AN4" s="51"/>
-      <c r="AO4" s="51"/>
-      <c r="AP4" s="51"/>
-      <c r="AQ4" s="51"/>
-      <c r="AR4" s="51"/>
-      <c r="AS4" s="51"/>
-      <c r="AT4" s="51"/>
-      <c r="AU4" s="51"/>
-      <c r="AV4" s="51"/>
-      <c r="AW4" s="51"/>
-      <c r="AX4" s="51"/>
-      <c r="AY4" s="51"/>
-      <c r="AZ4" s="51"/>
+      <c r="V4" s="51"/>
+      <c r="W4" s="51"/>
+      <c r="X4" s="44"/>
+      <c r="Y4" s="44"/>
+      <c r="Z4" s="44"/>
+      <c r="AA4" s="44"/>
+      <c r="AB4" s="44"/>
+      <c r="AC4" s="44"/>
+      <c r="AD4" s="44"/>
+      <c r="AE4" s="44"/>
+      <c r="AF4" s="44"/>
+      <c r="AG4" s="44"/>
+      <c r="AH4" s="58"/>
+      <c r="AI4" s="58"/>
+      <c r="AJ4" s="58"/>
+      <c r="AK4" s="58"/>
+      <c r="AL4" s="58"/>
+      <c r="AM4" s="58"/>
+      <c r="AN4" s="58"/>
+      <c r="AO4" s="58"/>
+      <c r="AP4" s="58"/>
+      <c r="AQ4" s="58"/>
+      <c r="AR4" s="58"/>
+      <c r="AS4" s="58"/>
+      <c r="AT4" s="58"/>
+      <c r="AU4" s="58"/>
+      <c r="AV4" s="58"/>
+      <c r="AW4" s="58"/>
+      <c r="AX4" s="58"/>
+      <c r="AY4" s="58"/>
+      <c r="AZ4" s="58"/>
     </row>
     <row r="5" spans="1:52" ht="26.4" thickBot="1">
       <c r="A5" s="32" t="s">
@@ -4186,19 +4186,19 @@
       <c r="E5" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="55" t="s">
+      <c r="F5" s="54" t="s">
         <v>115</v>
       </c>
-      <c r="G5" s="56"/>
+      <c r="G5" s="55"/>
       <c r="H5" s="31"/>
       <c r="I5" s="31"/>
       <c r="J5" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="K5" s="48">
+      <c r="K5" s="56">
         <v>0.5</v>
       </c>
-      <c r="L5" s="49"/>
+      <c r="L5" s="57"/>
       <c r="M5" s="31"/>
       <c r="N5" s="32" t="s">
         <v>5</v>
@@ -4256,10 +4256,10 @@
       <c r="A6" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="46">
+      <c r="B6" s="61">
         <v>46255</v>
       </c>
-      <c r="C6" s="47"/>
+      <c r="C6" s="62"/>
       <c r="D6" s="33"/>
       <c r="E6" s="33"/>
       <c r="F6" s="31"/>
@@ -4269,10 +4269,10 @@
       <c r="J6" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="K6" s="48">
+      <c r="K6" s="56">
         <v>2</v>
       </c>
-      <c r="L6" s="49"/>
+      <c r="L6" s="57"/>
       <c r="M6" s="31"/>
       <c r="N6" s="32" t="s">
         <v>9</v>
@@ -4334,7 +4334,7 @@
         <v>62.18</v>
       </c>
       <c r="C7" s="40">
-        <v>44.94</v>
+        <v>45</v>
       </c>
       <c r="D7" s="33"/>
       <c r="E7" s="33"/>
@@ -4397,7 +4397,7 @@
         <v>62.18</v>
       </c>
       <c r="C8" s="42">
-        <v>44.94</v>
+        <v>45</v>
       </c>
       <c r="D8" s="33"/>
       <c r="E8" s="33"/>
@@ -4724,70 +4724,70 @@
       <c r="F12" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="G12" s="44" t="s">
+      <c r="G12" s="59" t="s">
         <v>19</v>
       </c>
-      <c r="H12" s="44"/>
-      <c r="I12" s="44"/>
-      <c r="J12" s="44"/>
-      <c r="K12" s="44"/>
+      <c r="H12" s="59"/>
+      <c r="I12" s="59"/>
+      <c r="J12" s="59"/>
+      <c r="K12" s="59"/>
       <c r="L12" s="8" t="s">
         <v>20</v>
       </c>
       <c r="M12" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="N12" s="45" t="s">
+      <c r="N12" s="60" t="s">
         <v>22</v>
       </c>
-      <c r="O12" s="45"/>
-      <c r="P12" s="45"/>
-      <c r="Q12" s="45"/>
-      <c r="R12" s="50" t="s">
+      <c r="O12" s="60"/>
+      <c r="P12" s="60"/>
+      <c r="Q12" s="60"/>
+      <c r="R12" s="63" t="s">
         <v>23</v>
       </c>
-      <c r="S12" s="50"/>
-      <c r="T12" s="50"/>
-      <c r="U12" s="50"/>
-      <c r="V12" s="50"/>
-      <c r="W12" s="50"/>
-      <c r="X12" s="50"/>
-      <c r="Y12" s="50"/>
-      <c r="Z12" s="50"/>
-      <c r="AA12" s="44" t="s">
+      <c r="S12" s="63"/>
+      <c r="T12" s="63"/>
+      <c r="U12" s="63"/>
+      <c r="V12" s="63"/>
+      <c r="W12" s="63"/>
+      <c r="X12" s="63"/>
+      <c r="Y12" s="63"/>
+      <c r="Z12" s="63"/>
+      <c r="AA12" s="59" t="s">
         <v>24</v>
       </c>
-      <c r="AB12" s="44"/>
-      <c r="AC12" s="44"/>
-      <c r="AD12" s="44"/>
-      <c r="AE12" s="44" t="s">
+      <c r="AB12" s="59"/>
+      <c r="AC12" s="59"/>
+      <c r="AD12" s="59"/>
+      <c r="AE12" s="59" t="s">
         <v>25</v>
       </c>
-      <c r="AF12" s="44"/>
-      <c r="AG12" s="44"/>
-      <c r="AH12" s="44"/>
-      <c r="AI12" s="45" t="s">
+      <c r="AF12" s="59"/>
+      <c r="AG12" s="59"/>
+      <c r="AH12" s="59"/>
+      <c r="AI12" s="60" t="s">
         <v>26</v>
       </c>
-      <c r="AJ12" s="45"/>
-      <c r="AK12" s="45"/>
-      <c r="AL12" s="45"/>
-      <c r="AM12" s="45"/>
-      <c r="AN12" s="45"/>
-      <c r="AO12" s="45"/>
-      <c r="AP12" s="45"/>
-      <c r="AQ12" s="45"/>
-      <c r="AR12" s="45"/>
-      <c r="AS12" s="45"/>
-      <c r="AT12" s="45"/>
-      <c r="AU12" s="45"/>
-      <c r="AV12" s="45"/>
-      <c r="AW12" s="45"/>
-      <c r="AX12" s="45"/>
-      <c r="AY12" s="45" t="s">
+      <c r="AJ12" s="60"/>
+      <c r="AK12" s="60"/>
+      <c r="AL12" s="60"/>
+      <c r="AM12" s="60"/>
+      <c r="AN12" s="60"/>
+      <c r="AO12" s="60"/>
+      <c r="AP12" s="60"/>
+      <c r="AQ12" s="60"/>
+      <c r="AR12" s="60"/>
+      <c r="AS12" s="60"/>
+      <c r="AT12" s="60"/>
+      <c r="AU12" s="60"/>
+      <c r="AV12" s="60"/>
+      <c r="AW12" s="60"/>
+      <c r="AX12" s="60"/>
+      <c r="AY12" s="60" t="s">
         <v>27</v>
       </c>
-      <c r="AZ12" s="45"/>
+      <c r="AZ12" s="60"/>
     </row>
     <row r="13" spans="1:52" ht="15.6">
       <c r="A13" s="8"/>
@@ -6189,12 +6189,31 @@
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="Y3:Y4"/>
-    <mergeCell ref="A1:F2"/>
-    <mergeCell ref="G1:M2"/>
-    <mergeCell ref="V3:V4"/>
-    <mergeCell ref="W3:W4"/>
-    <mergeCell ref="X3:X4"/>
+    <mergeCell ref="AE12:AH12"/>
+    <mergeCell ref="AI12:AX12"/>
+    <mergeCell ref="AY12:AZ12"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="K6:L6"/>
+    <mergeCell ref="G12:K12"/>
+    <mergeCell ref="N12:Q12"/>
+    <mergeCell ref="R12:Z12"/>
+    <mergeCell ref="AA12:AD12"/>
+    <mergeCell ref="AX3:AX4"/>
+    <mergeCell ref="AY3:AY4"/>
+    <mergeCell ref="AZ3:AZ4"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="AT3:AT4"/>
+    <mergeCell ref="AU3:AU4"/>
+    <mergeCell ref="AV3:AV4"/>
+    <mergeCell ref="AW3:AW4"/>
+    <mergeCell ref="AK3:AK4"/>
+    <mergeCell ref="Z3:Z4"/>
+    <mergeCell ref="AA3:AA4"/>
+    <mergeCell ref="AB3:AB4"/>
+    <mergeCell ref="AC3:AC4"/>
+    <mergeCell ref="AD3:AD4"/>
+    <mergeCell ref="AE3:AE4"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="F5:G5"/>
     <mergeCell ref="K5:L5"/>
@@ -6211,31 +6230,12 @@
     <mergeCell ref="AH3:AH4"/>
     <mergeCell ref="AI3:AI4"/>
     <mergeCell ref="AJ3:AJ4"/>
-    <mergeCell ref="AX3:AX4"/>
-    <mergeCell ref="AY3:AY4"/>
-    <mergeCell ref="AZ3:AZ4"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="AT3:AT4"/>
-    <mergeCell ref="AU3:AU4"/>
-    <mergeCell ref="AV3:AV4"/>
-    <mergeCell ref="AW3:AW4"/>
-    <mergeCell ref="AK3:AK4"/>
-    <mergeCell ref="Z3:Z4"/>
-    <mergeCell ref="AA3:AA4"/>
-    <mergeCell ref="AB3:AB4"/>
-    <mergeCell ref="AC3:AC4"/>
-    <mergeCell ref="AD3:AD4"/>
-    <mergeCell ref="AE3:AE4"/>
-    <mergeCell ref="AE12:AH12"/>
-    <mergeCell ref="AI12:AX12"/>
-    <mergeCell ref="AY12:AZ12"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="K6:L6"/>
-    <mergeCell ref="G12:K12"/>
-    <mergeCell ref="N12:Q12"/>
-    <mergeCell ref="R12:Z12"/>
-    <mergeCell ref="AA12:AD12"/>
+    <mergeCell ref="Y3:Y4"/>
+    <mergeCell ref="A1:F2"/>
+    <mergeCell ref="G1:M2"/>
+    <mergeCell ref="V3:V4"/>
+    <mergeCell ref="W3:W4"/>
+    <mergeCell ref="X3:X4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>